<commit_message>
Working code - June 2nd morning
Working code - June 2nd morning
</commit_message>
<xml_diff>
--- a/Ref docs/Project Details.xlsx
+++ b/Ref docs/Project Details.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASharma33\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC79762-26E8-4166-938B-3DC1520AFDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{ECC79762-26E8-4166-938B-3DC1520AFDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{665F194F-DA46-4C52-9689-B4E36E76E982}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="751" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="SOW Budget -  ZS India" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SOW Budget -  ZS India'!$A$1:$U$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SOW Budget -  ZS India'!$A$1:$U$38</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="80">
   <si>
     <t>S.No.</t>
   </si>
@@ -300,6 +300,12 @@
   </si>
   <si>
     <t>ZSUS0376 - Mckesson Project 2026.</t>
+  </si>
+  <si>
+    <t>ZSUS0378 - Sanofi Projects 2026</t>
+  </si>
+  <si>
+    <t>Sanofi</t>
   </si>
 </sst>
 </file>
@@ -430,7 +436,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -603,12 +609,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -793,13 +812,37 @@
     </xf>
     <xf numFmtId="2" fontId="3" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1100,7 +1143,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="B1:U39"/>
+  <dimension ref="B1:U40"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" style="6" customWidth="1"/>
@@ -2972,65 +3015,119 @@
       <c r="T36" s="27"/>
       <c r="U36" s="27"/>
     </row>
-    <row r="37" spans="2:21" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="61">
+    <row r="37" spans="2:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="60">
         <v>36</v>
       </c>
-      <c r="C37" s="40" t="s">
+      <c r="C37" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="53" t="str">
+        <f>LEFT(C37,FIND(" ",C37)-1)</f>
+        <v>ZSUS0378</v>
+      </c>
+      <c r="E37" s="51" t="s">
+        <v>79</v>
+      </c>
+      <c r="F37" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="H37" s="26"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="26"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="27"/>
+      <c r="O37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="P37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="Q37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="R37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="S37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="T37" s="35">
+        <v>500923</v>
+      </c>
+      <c r="U37" s="35">
+        <v>500923</v>
+      </c>
+    </row>
+    <row r="38" spans="2:21" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B38" s="61">
+        <v>36</v>
+      </c>
+      <c r="C38" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="D37" s="54" t="str">
-        <f>LEFT(C37,FIND(" ",C37)-1)</f>
+      <c r="D38" s="54" t="str">
+        <f>LEFT(C38,FIND(" ",C38)-1)</f>
         <v>TBD</v>
       </c>
-      <c r="E37" s="52" t="s">
+      <c r="E38" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="F37" s="49" t="s">
+      <c r="F38" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="G37" s="36"/>
-      <c r="H37" s="36"/>
-      <c r="I37" s="36"/>
-      <c r="J37" s="36"/>
-      <c r="K37" s="36"/>
-      <c r="L37" s="36"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="38"/>
-      <c r="O37" s="38">
-        <v>500923</v>
-      </c>
-      <c r="P37" s="39"/>
-      <c r="Q37" s="39"/>
-      <c r="R37" s="39"/>
-      <c r="S37" s="39"/>
-      <c r="T37" s="37"/>
-      <c r="U37" s="37"/>
-    </row>
-    <row r="38" spans="2:21" ht="8" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="D39" s="1"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="20"/>
-      <c r="P39" s="20"/>
-      <c r="Q39" s="20"/>
-      <c r="R39" s="20"/>
-      <c r="S39" s="20"/>
-      <c r="T39" s="20"/>
-      <c r="U39" s="20"/>
+      <c r="G38" s="36"/>
+      <c r="H38" s="36"/>
+      <c r="I38" s="36"/>
+      <c r="J38" s="36"/>
+      <c r="K38" s="36"/>
+      <c r="L38" s="36"/>
+      <c r="M38" s="37"/>
+      <c r="N38" s="38"/>
+      <c r="O38" s="38">
+        <v>500923</v>
+      </c>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="39"/>
+      <c r="R38" s="39"/>
+      <c r="S38" s="39"/>
+      <c r="T38" s="37"/>
+      <c r="U38" s="37"/>
+    </row>
+    <row r="39" spans="2:21" ht="8" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="40" spans="2:21" x14ac:dyDescent="0.35">
+      <c r="D40" s="1"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
+      <c r="O40" s="20"/>
+      <c r="P40" s="20"/>
+      <c r="Q40" s="20"/>
+      <c r="R40" s="20"/>
+      <c r="S40" s="20"/>
+      <c r="T40" s="20"/>
+      <c r="U40" s="20"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="A1:U37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:U38" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="C37">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>